<commit_message>
checkpoint before auto fixes
Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/links.xlsx
+++ b/links.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\AeroESP\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9491C4A2-E6AB-4CBF-83F8-864E6F23818B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A840C54-38B2-4F0B-A209-BC7D904D9C60}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4704" yWindow="3396" windowWidth="17280" windowHeight="8964" xr2:uid="{ED9269C0-1221-42B0-9592-BDAAAC5F657A}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12576" xr2:uid="{ED9269C0-1221-42B0-9592-BDAAAC5F657A}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -34,7 +34,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="66" uniqueCount="66">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="69" uniqueCount="68">
   <si>
     <t>بخش</t>
   </si>
@@ -232,13 +232,19 @@
   </si>
   <si>
     <t>دستورات  cmd</t>
+  </si>
+  <si>
+    <t>cd /d D:\VTOLi</t>
+  </si>
+  <si>
+    <t>venv\Scripts\activate</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -260,6 +266,14 @@
       <name val="Arial Unicode MS"/>
       <family val="2"/>
     </font>
+    <font>
+      <u/>
+      <sz val="11"/>
+      <color theme="10"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -278,10 +292,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -292,8 +307,12 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -606,7 +625,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{0B24DC15-AF59-4743-A112-558D703BBB8C}">
-  <dimension ref="A1:B35"/>
+  <dimension ref="A1:B42"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="20" customWidth="1"/>
@@ -625,7 +644,7 @@
       <c r="A2" s="2" t="s">
         <v>2</v>
       </c>
-      <c r="B2" s="3" t="s">
+      <c r="B2" s="4" t="s">
         <v>3</v>
       </c>
     </row>
@@ -881,7 +900,25 @@
         <v>64</v>
       </c>
     </row>
+    <row r="40" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B40" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="41" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B41" t="s">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="42" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B42" t="s">
+        <v>62</v>
+      </c>
+    </row>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B2" r:id="rId1" xr:uid="{1D26B14E-ED9B-4A7A-8C58-E682EDC6454F}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>